<commit_message>
Add GameData snapshot, meal proposals and Google Sheet tooling
- .gitignore: never commit the Google service account key
- simulate/tools/gsheet.py: read/write the Sumeeper_GameData sheet Unity loads
- simulate/tools/meal_stat.py
- game_document/Sumeeper_GameData.xlsx: snapshot of that sheet
- game_document/proposals/: MealItem names, MealStat, RecipeItem alignment
- Sumeeper_Meal_Sheet.xlsx updates

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/game_document/Sumeeper_Meal_Sheet.xlsx
+++ b/game_document/Sumeeper_Meal_Sheet.xlsx
@@ -14,21 +14,21 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
+    <t>Sumeeper — Meal Effect (สูตรอาหารในดันเจี้ยน)</t>
+  </si>
+  <si>
     <t>Sumeeper — Meal Effect Reference Sheet</t>
   </si>
   <si>
-    <t>Sumeeper — Meal Effect (สูตรอาหารในดันเจี้ยน)</t>
-  </si>
-  <si>
     <t>สรุประบบ Meal Effect — จัดทำจาก "sumeeper data" Google ชีต (แท็บ Meal Effect)</t>
   </si>
   <si>
+    <t>ยิ่งใช้ Seasoning มาก Restore ยิ่งต่ำแต่ได้ Effect พิเศษแรงขึ้น</t>
+  </si>
+  <si>
     <t>โครงสร้างวัตถุดิบ (Ingredient Code)</t>
   </si>
   <si>
-    <t>ยิ่งใช้ Seasoning มาก Restore ยิ่งต่ำแต่ได้ Effect พิเศษแรงขึ้น</t>
-  </si>
-  <si>
     <t>m</t>
   </si>
   <si>
@@ -59,34 +59,34 @@
     <t>Ingredients</t>
   </si>
   <si>
+    <t>Code</t>
+  </si>
+  <si>
     <t>6 สูตร — Meat/Vegie/Seasoning ผสมกัน 2 ชนิด (รวมซ้ำได้ เช่น mm)</t>
   </si>
   <si>
+    <t>Restore HP</t>
+  </si>
+  <si>
     <t>3-Ingredient Meal</t>
   </si>
   <si>
-    <t>Code</t>
-  </si>
-  <si>
     <t>10 สูตร — ผสมกัน 3 ชนิด (รวมซ้ำได้ เช่น mmm, sss)</t>
   </si>
   <si>
+    <t>Max HP</t>
+  </si>
+  <si>
     <t>Restore Health / Stamina</t>
   </si>
   <si>
+    <t>Restore Stamina</t>
+  </si>
+  <si>
+    <t>Effect</t>
+  </si>
+  <si>
     <t>ยิ่งเนื้อ (Meat) เยอะ ค่า Restore ยิ่งสูง; ยิ่ง Seasoning เยอะ ค่า Restore ยิ่งต่ำ (เทรดกับ Effect ที่แรงขึ้น)</t>
-  </si>
-  <si>
-    <t>Max HP</t>
-  </si>
-  <si>
-    <t>Restore HP</t>
-  </si>
-  <si>
-    <t>Restore Stamina</t>
-  </si>
-  <si>
-    <t>Effect</t>
   </si>
   <si>
     <t>2-Ingredient Meals (6 สูตร)</t>
@@ -300,13 +300,13 @@
     </font>
     <font>
       <b/>
-      <sz val="18.0"/>
+      <sz val="16.0"/>
       <color rgb="FF7A3B1E"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="18.0"/>
       <color rgb="FF7A3B1E"/>
       <name val="Arial"/>
     </font>
@@ -345,7 +345,6 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <b/>
       <sz val="11.0"/>
@@ -362,6 +361,10 @@
       <b/>
       <sz val="10.0"/>
       <color rgb="FFB33F00"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -447,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -478,37 +481,47 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="1" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -739,8 +752,8 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
@@ -750,7 +763,7 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -787,23 +800,23 @@
         <v>13</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1814,14 +1827,26 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>4</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
@@ -1831,19 +1856,19 @@
         <v>14</v>
       </c>
       <c r="C4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>21</v>
-      </c>
       <c r="E4" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" ht="19.5" customHeight="1">
@@ -1871,10 +1896,10 @@
         <v>6.0</v>
       </c>
       <c r="E6" s="17">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
       <c r="F6" s="17">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>29</v>
@@ -1894,14 +1919,17 @@
         <v>4.0</v>
       </c>
       <c r="E7" s="17">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="F7" s="17">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>33</v>
       </c>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
     </row>
     <row r="8" ht="33.75" customHeight="1">
       <c r="A8" s="14" t="s">
@@ -1917,14 +1945,17 @@
         <v>3.0</v>
       </c>
       <c r="E8" s="17">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F8" s="17">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>37</v>
       </c>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
     </row>
     <row r="9" ht="33.75" customHeight="1">
       <c r="A9" s="14" t="s">
@@ -1940,14 +1971,17 @@
         <v>2.0</v>
       </c>
       <c r="E9" s="17">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="F9" s="17">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>41</v>
       </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
     </row>
     <row r="10" ht="33.75" customHeight="1">
       <c r="A10" s="14" t="s">
@@ -1963,14 +1997,17 @@
         <v>1.0</v>
       </c>
       <c r="E10" s="17">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="F10" s="17">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>45</v>
       </c>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
     </row>
     <row r="11" ht="33.75" customHeight="1">
       <c r="A11" s="14" t="s">
@@ -1986,7 +2023,7 @@
         <v>0.0</v>
       </c>
       <c r="E11" s="17">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="F11" s="17">
         <v>0.0</v>
@@ -1994,6 +2031,9 @@
       <c r="G11" s="15" t="s">
         <v>49</v>
       </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" s="11" t="s">
@@ -2005,234 +2045,240 @@
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
       <c r="G12" s="13"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
     </row>
     <row r="13" ht="33.75" customHeight="1">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="23">
         <v>9.0</v>
       </c>
-      <c r="E13" s="21">
-        <v>9.0</v>
-      </c>
-      <c r="F13" s="21">
-        <v>9.0</v>
-      </c>
-      <c r="G13" s="19" t="s">
+      <c r="E13" s="23">
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="G13" s="21" t="s">
         <v>54</v>
       </c>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
     </row>
     <row r="14" ht="33.75" customHeight="1">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="23">
         <v>7.0</v>
       </c>
-      <c r="E14" s="21">
-        <v>7.0</v>
-      </c>
-      <c r="F14" s="21">
-        <v>7.0</v>
-      </c>
-      <c r="G14" s="19" t="s">
+      <c r="E14" s="23">
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G14" s="21" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" ht="33.75" customHeight="1">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="23">
         <v>6.0</v>
       </c>
-      <c r="E15" s="21">
-        <v>6.0</v>
-      </c>
-      <c r="F15" s="21">
-        <v>6.0</v>
-      </c>
-      <c r="G15" s="19" t="s">
+      <c r="E15" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="F15" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="G15" s="21" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="16" ht="33.75" customHeight="1">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="23">
         <v>5.0</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="23">
+        <v>0.0</v>
+      </c>
+      <c r="F16" s="23">
         <v>5.0</v>
       </c>
-      <c r="F16" s="21">
-        <v>5.0</v>
-      </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="21" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="17" ht="33.75" customHeight="1">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="21">
+      <c r="D17" s="23">
         <v>4.0</v>
       </c>
-      <c r="E17" s="21">
-        <v>4.0</v>
-      </c>
-      <c r="F17" s="21">
-        <v>4.0</v>
-      </c>
-      <c r="G17" s="19" t="s">
+      <c r="E17" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="F17" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="G17" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="18" ht="33.75" customHeight="1">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="23">
         <v>3.0</v>
       </c>
-      <c r="E18" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="F18" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="G18" s="19" t="s">
+      <c r="E18" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="F18" s="23">
+        <v>1.0</v>
+      </c>
+      <c r="G18" s="21" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="19" ht="33.75" customHeight="1">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="23">
         <v>3.0</v>
       </c>
-      <c r="E19" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="F19" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="G19" s="19" t="s">
+      <c r="E19" s="23">
+        <v>0.0</v>
+      </c>
+      <c r="F19" s="23">
+        <v>6.0</v>
+      </c>
+      <c r="G19" s="21" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="20" ht="33.75" customHeight="1">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="21">
+      <c r="D20" s="23">
         <v>2.0</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="23">
         <v>2.0</v>
       </c>
-      <c r="F20" s="21">
-        <v>2.0</v>
-      </c>
-      <c r="G20" s="19" t="s">
+      <c r="F20" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G20" s="21" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="21" ht="33.75" customHeight="1">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="23">
         <v>1.0</v>
       </c>
-      <c r="E21" s="21">
-        <v>1.0</v>
-      </c>
-      <c r="F21" s="21">
-        <v>1.0</v>
-      </c>
-      <c r="G21" s="19" t="s">
+      <c r="E21" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="F21" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="G21" s="21" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="23">
         <v>0.0</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="23">
+        <v>6.0</v>
+      </c>
+      <c r="F22" s="23">
         <v>0.0</v>
       </c>
-      <c r="F22" s="21">
-        <v>0.0</v>
-      </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="21" t="s">
         <v>90</v>
       </c>
     </row>
@@ -3215,12 +3261,6 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A12:G12"/>
-  </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>